<commit_message>
Corrección formatos y logos
</commit_message>
<xml_diff>
--- a/backend/src/main/resources/reports/bitacora-template.xlsx
+++ b/backend/src/main/resources/reports/bitacora-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Personal\SistemaTrafico\EcuTrans9000\backend\src\main\resources\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86F0D10A-5329-4A7C-B5C6-C051B8D104B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32515379-DFD1-4EA2-A9FE-BF7E282D0E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-35700" yWindow="2700" windowWidth="28800" windowHeight="11235" xr2:uid="{69F4AFB3-3EC8-44DE-B7BA-26A03C1E8902}"/>
+    <workbookView xWindow="-31920" yWindow="2415" windowWidth="24120" windowHeight="11235" xr2:uid="{69F4AFB3-3EC8-44DE-B7BA-26A03C1E8902}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -144,15 +144,15 @@
     <t xml:space="preserve">Anticipo </t>
   </si>
   <si>
-    <t>Facturado
-Cliente</t>
-  </si>
-  <si>
     <t>Pagado
 transportista</t>
   </si>
   <si>
     <t>Fecha Pago Cliente a Ecutrans</t>
+  </si>
+  <si>
+    <t>Pagado
+Cliente</t>
   </si>
 </sst>
 </file>
@@ -718,7 +718,7 @@
         <v>34</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N7" s="1" t="s">
         <v>26</v>
@@ -727,10 +727,10 @@
         <v>27</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="R7" s="10"/>
       <c r="S7" s="10"/>

</xml_diff>

<commit_message>
lógica combo Destino según lista de equivalencia de precios
</commit_message>
<xml_diff>
--- a/backend/src/main/resources/reports/bitacora-template.xlsx
+++ b/backend/src/main/resources/reports/bitacora-template.xlsx
@@ -639,7 +639,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABA269E4-D87E-4FE1-BA98-39DF1C5A346E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{ABA269E4-D87E-4FE1-BA98-39DF1C5A346E}">
   <dimension ref="A4:S10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
@@ -732,7 +732,11 @@
       <c r="Q7" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="R7" s="10"/>
+      <c r="R7" s="10" t="inlineStr">
+        <is>
+          <t>Costo Chofer</t>
+        </is>
+      </c>
       <c r="S7" s="10"/>
     </row>
     <row r="8" spans="1:19">
@@ -895,12 +899,12 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A7:Q7" xr:uid="{ABA269E4-D87E-4FE1-BA98-39DF1C5A346E}"/>
+  <autoFilter ref="A7:Q7" ns2:uid="{ABA269E4-D87E-4FE1-BA98-39DF1C5A346E}"/>
   <mergeCells count="1">
     <mergeCell ref="A4:Q4"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <drawing ns3:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>